<commit_message>
Sistemato generazione file dati base
sistemato la generazione dle file in modo che il progetto compila e fatto maggiori divisioni per i difetti
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4B_Risultati_GridSearch_MLP.xlsx
+++ b/export_dati/04_Step4B_Risultati_GridSearch_MLP.xlsx
@@ -456,28 +456,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>0.01</v>
       </c>
       <c r="D2" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>98.98%</t>
+          <t>93.97%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -492,7 +492,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -503,43 +503,43 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>98.73%</t>
+          <t>93.97%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>98.72%</t>
+          <t>93.93%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.0014</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -554,23 +554,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>98.72%</t>
+          <t>93.93%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.0005</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -596,12 +596,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>98.70%</t>
+          <t>93.92%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.0015</t>
+          <t>0.0012</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -616,23 +616,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D7" t="n">
         <v>0.0001</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>98.68%</t>
+          <t>93.73%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.0015</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -642,43 +642,43 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>0.001</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>98.62%</t>
+          <t>93.73%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.0006</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -689,12 +689,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>98.57%</t>
+          <t>93.68%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>0.0026</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -709,23 +709,23 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>0.001</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>98.55%</t>
+          <t>93.67%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.0018</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -747,16 +747,16 @@
         <v>0.001</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>98.55%</t>
+          <t>93.67%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.0015</t>
+          <t>0.0018</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -766,28 +766,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>0.01</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>98.53%</t>
+          <t>93.63%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.0009</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -797,28 +797,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D13" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>98.53%</t>
+          <t>93.63%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.0019</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -828,12 +828,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -844,43 +844,43 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>98.53%</t>
+          <t>93.62%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.0040</t>
+          <t>0.0035</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>0.01</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>98.52%</t>
+          <t>93.60%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>0.0037</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -906,22 +906,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>98.48%</t>
+          <t>93.60%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.0006</t>
+          <t>0.0044</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -930,19 +930,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D17" t="n">
         <v>0.0001</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>98.43%</t>
+          <t>93.58%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.0017</t>
+          <t>0.0044</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -952,28 +952,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>0.001</v>
       </c>
       <c r="D18" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>98.43%</t>
+          <t>93.57%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.0051</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -988,7 +988,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -999,12 +999,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>98.37%</t>
+          <t>93.55%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.0015</t>
+          <t>0.0025</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1014,7 +1014,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1030,12 +1030,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>98.35%</t>
+          <t>93.55%</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.0015</t>
+          <t>0.0050</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1057,16 +1057,16 @@
         <v>0.01</v>
       </c>
       <c r="D21" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>98.33%</t>
+          <t>93.50%</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.0011</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1076,28 +1076,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>98.30%</t>
+          <t>93.48%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.0057</t>
+          <t>0.0020</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1107,7 +1107,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1123,12 +1123,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>98.30%</t>
+          <t>93.48%</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.0057</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1138,7 +1138,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1150,16 +1150,16 @@
         <v>0.001</v>
       </c>
       <c r="D24" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>98.08%</t>
+          <t>93.22%</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0.0046</t>
+          <t>0.0038</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1169,7 +1169,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1181,20 +1181,20 @@
         <v>0.001</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>98.03%</t>
+          <t>93.22%</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0.0042</t>
+          <t>0.0038</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sistemato funzionamento con 1 sola barra per entrambi i test
Sistemato codice in modo da usare una sola barra per entrambi i check in modo da poter fare il confronto inoltre c'era un problema nella generazione dle file
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4B_Risultati_GridSearch_MLP.xlsx
+++ b/export_dati/04_Step4B_Risultati_GridSearch_MLP.xlsx
@@ -456,12 +456,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -472,12 +472,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>93.97%</t>
+          <t>96.10%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>0.0008</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -503,22 +503,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>93.97%</t>
+          <t>96.05%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>0.0014</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -527,19 +527,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D4" t="n">
         <v>0.01</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>93.93%</t>
+          <t>95.98%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>0.0008</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -549,38 +549,38 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D5" t="n">
         <v>0.0001</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>93.93%</t>
+          <t>95.92%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>0.0029</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -596,12 +596,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>93.92%</t>
+          <t>95.83%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.0012</t>
+          <t>0.0008</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -611,12 +611,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -627,16 +627,16 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>93.73%</t>
+          <t>95.83%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>0.0006</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -647,33 +647,33 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>93.73%</t>
+          <t>95.82%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>0.0006</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -682,29 +682,29 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>93.68%</t>
+          <t>95.82%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.0026</t>
+          <t>0.0006</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -713,29 +713,29 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>93.67%</t>
+          <t>95.82%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.0014</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -744,29 +744,29 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D11" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>93.67%</t>
+          <t>95.82%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.0014</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -778,16 +778,16 @@
         <v>0.01</v>
       </c>
       <c r="D12" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>93.63%</t>
+          <t>95.75%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>0.0019</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -809,26 +809,26 @@
         <v>0.01</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>93.63%</t>
+          <t>95.73%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>0.0019</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -840,26 +840,26 @@
         <v>0.01</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>93.62%</t>
+          <t>95.73%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.0035</t>
+          <t>0.0013</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -868,19 +868,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>93.60%</t>
+          <t>95.72%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.0037</t>
+          <t>0.0025</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -899,19 +899,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D16" t="n">
         <v>0.01</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>93.60%</t>
+          <t>95.72%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.0044</t>
+          <t>0.0025</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -937,12 +937,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>93.58%</t>
+          <t>95.67%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.0044</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -952,7 +952,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -968,12 +968,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>93.57%</t>
+          <t>95.57%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.0051</t>
+          <t>0.0022</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -983,23 +983,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>0.001</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>93.55%</t>
+          <t>95.55%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1014,7 +1014,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1030,12 +1030,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>93.55%</t>
+          <t>95.30%</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.0050</t>
+          <t>0.0023</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1045,59 +1045,59 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D21" t="n">
         <v>0.0001</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>93.50%</t>
+          <t>95.30%</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0.0011</t>
+          <t>0.0051</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D22" t="n">
         <v>0.01</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>93.48%</t>
+          <t>95.28%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.0020</t>
+          <t>0.0051</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1107,7 +1107,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1119,16 +1119,16 @@
         <v>0.001</v>
       </c>
       <c r="D23" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>93.48%</t>
+          <t>95.28%</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>0.0065</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1138,28 +1138,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>0.001</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>93.22%</t>
+          <t>95.27%</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0.0038</t>
+          <t>0.0065</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1181,20 +1181,20 @@
         <v>0.001</v>
       </c>
       <c r="D25" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>93.22%</t>
+          <t>95.23%</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0.0038</t>
+          <t>0.0014</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test su 100 barre on statistiche
Fatto il loop per fare i test su 100 barre e fare le statistiche,
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4B_Risultati_GridSearch_MLP.xlsx
+++ b/export_dati/04_Step4B_Risultati_GridSearch_MLP.xlsx
@@ -456,28 +456,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>0.01</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>96.10%</t>
+          <t>95.92%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -487,7 +487,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -499,16 +499,16 @@
         <v>0.01</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>96.05%</t>
+          <t>95.87%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.0014</t>
+          <t>0.0012</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -518,7 +518,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -534,12 +534,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>95.98%</t>
+          <t>95.83%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -549,12 +549,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -565,43 +565,43 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>95.92%</t>
+          <t>95.83%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.0029</t>
+          <t>0.0012</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>0.01</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>95.83%</t>
+          <t>95.65%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.0032</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -616,23 +616,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>95.83%</t>
+          <t>95.65%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.0006</t>
+          <t>0.0032</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -642,7 +642,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -651,23 +651,23 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>95.82%</t>
+          <t>95.65%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.0006</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -685,26 +685,26 @@
         <v>0.001</v>
       </c>
       <c r="D9" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>95.82%</t>
+          <t>95.60%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.0006</t>
+          <t>0.0018</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -713,29 +713,29 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D10" t="n">
         <v>0.01</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>95.82%</t>
+          <t>95.57%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.0014</t>
+          <t>0.0024</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -744,23 +744,23 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D11" t="n">
         <v>0.0001</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>95.82%</t>
+          <t>95.55%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0.0014</t>
+          <t>0.0025</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -771,23 +771,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>0.01</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>95.75%</t>
+          <t>95.55%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.0019</t>
+          <t>0.0025</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -802,27 +802,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>0.01</v>
       </c>
       <c r="D13" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>95.73%</t>
+          <t>95.55%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.0019</t>
+          <t>0.0025</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -833,7 +833,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -844,43 +844,43 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>95.73%</t>
+          <t>95.53%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.0013</t>
+          <t>0.0030</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>95.72%</t>
+          <t>95.53%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.0025</t>
+          <t>0.0039</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -890,43 +890,43 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>0.001</v>
       </c>
       <c r="D16" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>95.72%</t>
+          <t>95.52%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.0025</t>
+          <t>0.0033</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -937,22 +937,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>95.67%</t>
+          <t>95.52%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>0.0039</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -964,16 +964,16 @@
         <v>0.001</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>95.57%</t>
+          <t>95.50%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.0022</t>
+          <t>0.0031</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -983,7 +983,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50, 25)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -992,19 +992,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D19" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>95.55%</t>
+          <t>95.47%</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.0025</t>
+          <t>0.0027</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1014,19 +1014,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>0.001</v>
       </c>
       <c r="D20" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.0023</t>
+          <t>0.0035</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1045,7 +1045,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1057,20 +1057,20 @@
         <v>0.001</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>95.30%</t>
+          <t>95.28%</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0.0051</t>
+          <t>0.0033</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -1088,16 +1088,16 @@
         <v>0.001</v>
       </c>
       <c r="D22" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>95.28%</t>
+          <t>95.10%</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.0051</t>
+          <t>0.0043</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1107,7 +1107,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>(100,)</t>
+          <t>(50,)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1119,20 +1119,20 @@
         <v>0.001</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>95.28%</t>
+          <t>95.08%</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.0065</t>
+          <t>0.0044</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1154,12 +1154,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>95.27%</t>
+          <t>94.87%</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0.0065</t>
+          <t>0.0059</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1169,7 +1169,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(100,)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1185,16 +1185,16 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>95.23%</t>
+          <t>94.87%</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0.0014</t>
+          <t>0.0059</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>